<commit_message>
Move filter dropdowns below headers on dashboard and comparison report pages
Layout Changes:
- Moved Project Coach and Project Name dropdowns below page headers
- Created separate filter container cards for better visual separation
- Updated CSS for both dashboard and comparison report pages

Styling Updates:
- Filter container now has its own white card with padding and shadow
- Header section reduced bottom margin to 1.5rem
- Filter container has 1.5rem vertical padding and 2rem horizontal padding
- Maintains consistent styling across both pages

Benefits:
- Cleaner visual hierarchy with title and filters separated
- More horizontal space for filter dropdowns
- Better mobile responsiveness
- Professional card-based design
- Improved user experience with dedicated filter section
</commit_message>
<xml_diff>
--- a/forecast_dummy.xlsx
+++ b/forecast_dummy.xlsx
@@ -1288,13 +1288,13 @@
         </is>
       </c>
       <c r="G2" s="8" t="n">
-        <v>20</v>
+        <v>2000</v>
       </c>
       <c r="H2" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>64.51600000000001</v>
+        <v>1000</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>140</v>
@@ -1324,13 +1324,13 @@
         <v>17</v>
       </c>
       <c r="S2" s="10" t="n">
-        <v>1120</v>
+        <v>3100</v>
       </c>
       <c r="T2" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U2" s="10" t="n">
-        <v>218.132</v>
+        <v>1153.616</v>
       </c>
       <c r="V2" s="10" t="n">
         <v>172</v>

</xml_diff>